<commit_message>
feat(generator): REQ-002 refined from product owner answers
- REQ-002 acceptance criteria 2-7, 9, 10 from the answers in review/questions/REQ-002.md
  (title rules, inclusive limit, dot decimal, categories, dates, duplicates, success
  message lifetime, same-date order); questions marked Resolved
- 23 new REQ-002 drafts (scenarios 25-42) and 19 "covered by existing test" rows

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requirements/expenses.xlsx
+++ b/requirements/expenses.xlsx
@@ -67,8 +67,15 @@
   </si>
   <si>
     <t xml:space="preserve">Title, amount, category and date are required
-Amount must be &gt; 0, at most 1,000,000, max 2 decimals
-Success message and the new row appear in the list</t>
+A whitespace-only title counts as missing; title is at most 200 characters
+Amount must be &gt; 0, at most 1,000,000 (inclusive), max 2 decimals
+Amount uses a dot decimal (12.50); no thousands separator
+Category is one of: Food, Travel, Office, Utilities, Entertainment, Other
+Date is any real date in YYYY-MM-DD format; future dates are allowed
+Duplicate expenses (same title, amount, category and date) are allowed
+Success message and the new row appear in the list
+The success message stays until the user opens Add or Edit or another message (e.g. an error) replaces it; filtering, Export and Import keep it
+The new row follows the date sort (newest first); on the same date the newest expense (higher id) comes first</t>
   </si>
   <si>
     <t>BUG-002, BUG-004</t>

</xml_diff>

<commit_message>
fix(api): enforce expense ownership by role (BUG-001, REQ-008)
A regular user reads and writes only their own expenses; another user's
returns 404. The admin reads every expense (list, export, GET by id) but
edits and deletes only their own; another user's returns 403.

- Remove the 8 BUG-001 test.fail() markers; tighten user checks to 404
- Add admin API and DB tests (read 200, list/export include, PUT/DELETE 403)
- REQ-008: Q1/Q2 resolved, acceptance criteria, drafts and traceability
- docs: BUG-001 fixed, BUG-005 (admin sees Edit/Delete on others' rows)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requirements/expenses.xlsx
+++ b/requirements/expenses.xlsx
@@ -159,11 +159,13 @@
     <t>As a user I want only my own expenses visible</t>
   </si>
   <si>
-    <t xml:space="preserve">The list, export and detail views show only my expenses
-I cannot edit or delete another user's expense</t>
-  </si>
-  <si>
-    <t>BUG-001</t>
+    <t xml:space="preserve">A regular user sees only their own expenses in the list, export and detail views; another user's expense returns 404
+A regular user cannot edit or delete another user's expense (404)
+The admin can view every user's expenses (list, export, detail)
+The admin can edit and delete only their own expenses; another user's returns 403</t>
+  </si>
+  <si>
+    <t>BUG-001, BUG-005</t>
   </si>
   <si>
     <t>REQ-009</t>

</xml_diff>

<commit_message>
feat: change-impact analysis (/analyze-change)
Map changed files to requirements, tests and risk for a branch, PR or
commit range.

- requirements/expenses.xlsx: new "Code map" sheet (42 rows: glob,
  requirement IDs or ALL, risk, fallback specs, notes), built by
  scripts/build-requirements.mts
- scripts/analyze-change.mts (npm run analyze:change): git diff, Code map
  match, tests via review/traceability.xlsx or fallback specs; any High row
  runs the full suite, smoke always runs, unmapped files warn; report also
  written to reports/change-impact.md
- /analyze-change skill wraps the script
- docs/examples/change-impact-bug-001.md: report for the BUG-001 fix

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requirements/expenses.xlsx
+++ b/requirements/expenses.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Requirements" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Code map" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="153">
   <si>
     <t>ID</t>
   </si>
@@ -198,6 +199,308 @@
   <si>
     <t xml:space="preserve">The list shows a total for the current month
 The total updates after add, edit or delete</t>
+  </si>
+  <si>
+    <t>Code path pattern</t>
+  </si>
+  <si>
+    <t>Requirement IDs</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>Fallback specs</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>app/api/src/app.js</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>Middleware: JSON limit, route wiring, /api 404, error handler (400/500)</t>
+  </si>
+  <si>
+    <t>app/api/src/server.js</t>
+  </si>
+  <si>
+    <t>API startup</t>
+  </si>
+  <si>
+    <t>app/api/src/db.js</t>
+  </si>
+  <si>
+    <t>pg pool; DATE and NUMERIC type parsers used by every read</t>
+  </si>
+  <si>
+    <t>app/api/src/auth.js</t>
+  </si>
+  <si>
+    <t>JWT sign/verify, requireAuth on every /api/expenses route; role used by REQ-008</t>
+  </si>
+  <si>
+    <t>app/api/src/routes/auth.js</t>
+  </si>
+  <si>
+    <t>POST /api/auth/login; every test logs in through it</t>
+  </si>
+  <si>
+    <t>app/api/src/validate.js</t>
+  </si>
+  <si>
+    <t>REQ-002, REQ-003, REQ-007</t>
+  </si>
+  <si>
+    <t>Shared expense validator for CRUD and xlsx import</t>
+  </si>
+  <si>
+    <t>app/api/src/routes/expenses.js</t>
+  </si>
+  <si>
+    <t>REQ-002, REQ-003, REQ-004, REQ-005, REQ-006, REQ-007, REQ-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/api/expenses.spec.ts
+tests/api/expenses-file.spec.ts
+tests/db/expenses.spec.ts
+tests/db/expenses-import.spec.ts
+tests/ui/expense-crud.spec.ts
+tests/ui/expense-list.spec.ts
+tests/ui/expense-files.spec.ts</t>
+  </si>
+  <si>
+    <t>CRUD, ?category filter, /export, /import, ownership checks (REQ-008)</t>
+  </si>
+  <si>
+    <t>app/api/*</t>
+  </si>
+  <si>
+    <t>package.json, lockfile, Dockerfile: dependencies and runtime</t>
+  </si>
+  <si>
+    <t>app/web/src/api.js</t>
+  </si>
+  <si>
+    <t>Shared fetch client, Bearer token, localStorage session, 401 handler</t>
+  </si>
+  <si>
+    <t>app/web/src/App.jsx</t>
+  </si>
+  <si>
+    <t>Session routing between Login and Expenses</t>
+  </si>
+  <si>
+    <t>app/web/src/main.jsx</t>
+  </si>
+  <si>
+    <t>Web entry point</t>
+  </si>
+  <si>
+    <t>app/web/src/pages/LoginPage.jsx</t>
+  </si>
+  <si>
+    <t>tests/ui/login.spec.ts</t>
+  </si>
+  <si>
+    <t>Login form and errors, session-expired notice</t>
+  </si>
+  <si>
+    <t>app/web/src/pages/ExpensesPage.jsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/ui/expense-crud.spec.ts
+tests/ui/expense-list.spec.ts
+tests/ui/expense-files.spec.ts</t>
+  </si>
+  <si>
+    <t>List, sort, filter, delete confirm, export/import, messages; REQ-009/010 will land here</t>
+  </si>
+  <si>
+    <t>app/web/src/components/ExpenseForm.jsx</t>
+  </si>
+  <si>
+    <t>REQ-002, REQ-003</t>
+  </si>
+  <si>
+    <t>tests/ui/expense-crud.spec.ts</t>
+  </si>
+  <si>
+    <t>Add/Edit form, client-side validation</t>
+  </si>
+  <si>
+    <t>app/web/src/styles.css</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Visual only; smoke covers it</t>
+  </si>
+  <si>
+    <t>app/web/*</t>
+  </si>
+  <si>
+    <t>nginx.conf (/api proxy), vite.config.js, index.html, Dockerfile, package files</t>
+  </si>
+  <si>
+    <t>app/db/init/01-schema.sql</t>
+  </si>
+  <si>
+    <t>Tables and constraints; needs a reseed (down -v)</t>
+  </si>
+  <si>
+    <t>app/db/init/02-seed.sql</t>
+  </si>
+  <si>
+    <t>Seed users and 20 expenses that tests count on; needs a reseed (down -v)</t>
+  </si>
+  <si>
+    <t>docker-compose.yml</t>
+  </si>
+  <si>
+    <t>Service wiring, env, ports</t>
+  </si>
+  <si>
+    <t>playwright.config.ts</t>
+  </si>
+  <si>
+    <t>Test projects, baseURLs, reporters</t>
+  </si>
+  <si>
+    <t>fixtures/**</t>
+  </si>
+  <si>
+    <t>Shared test fixtures and upload files</t>
+  </si>
+  <si>
+    <t>pages/**</t>
+  </si>
+  <si>
+    <t>Page objects used by every UI test</t>
+  </si>
+  <si>
+    <t>schemas/**</t>
+  </si>
+  <si>
+    <t>ajv response schemas</t>
+  </si>
+  <si>
+    <t>tests/auth.setup.ts</t>
+  </si>
+  <si>
+    <t>UI login state for the ui project</t>
+  </si>
+  <si>
+    <t>tests/db/db.helper.ts</t>
+  </si>
+  <si>
+    <t>Shared DB query helpers</t>
+  </si>
+  <si>
+    <t>tests/**/*.spec.ts</t>
+  </si>
+  <si>
+    <t>The changed spec itself is added to the run</t>
+  </si>
+  <si>
+    <t>package.json</t>
+  </si>
+  <si>
+    <t>Test dependencies and scripts</t>
+  </si>
+  <si>
+    <t>package-lock.json</t>
+  </si>
+  <si>
+    <t>Locked versions; also sets the Playwright image version</t>
+  </si>
+  <si>
+    <t>.nvmrc</t>
+  </si>
+  <si>
+    <t>Node version for local runs and CI</t>
+  </si>
+  <si>
+    <t>tests.Dockerfile</t>
+  </si>
+  <si>
+    <t>Docker test runner; verify with npm run test:docker:smoke</t>
+  </si>
+  <si>
+    <t>.github/**</t>
+  </si>
+  <si>
+    <t>CI workflow; verify on the PR run</t>
+  </si>
+  <si>
+    <t>review/**</t>
+  </si>
+  <si>
+    <t>AI drafts, not in the suite (optional review run)</t>
+  </si>
+  <si>
+    <t>requirements/**</t>
+  </si>
+  <si>
+    <t>Requirements data; check traceability is still in sync</t>
+  </si>
+  <si>
+    <t>scripts/**</t>
+  </si>
+  <si>
+    <t>Tooling; run the changed script</t>
+  </si>
+  <si>
+    <t>reporting/**</t>
+  </si>
+  <si>
+    <t>Excel report, CI summary, n8n payload</t>
+  </si>
+  <si>
+    <t>Jenkinsfile</t>
+  </si>
+  <si>
+    <t>Nightly pipeline</t>
+  </si>
+  <si>
+    <t>jenkins/**</t>
+  </si>
+  <si>
+    <t>Local Jenkins stack</t>
+  </si>
+  <si>
+    <t>n8n/**</t>
+  </si>
+  <si>
+    <t>Failure-to-Jira workflow</t>
+  </si>
+  <si>
+    <t>.claude/**</t>
+  </si>
+  <si>
+    <t>Skills and settings</t>
+  </si>
+  <si>
+    <t>**/*.md</t>
+  </si>
+  <si>
+    <t>Docs (CLAUDE.md, docs/, READMEs)</t>
+  </si>
+  <si>
+    <t>.env.example</t>
+  </si>
+  <si>
+    <t>Demo config template, no secrets</t>
+  </si>
+  <si>
+    <t>.gitignore</t>
+  </si>
+  <si>
+    <t>Repo hygiene</t>
   </si>
 </sst>
 </file>
@@ -852,4 +1155,752 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E43"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>